<commit_message>
docs(catalog): add IRIB production drinks to final price list
Include 38 new IRIB SKUs and 11 existing ZY-IRIB items as a separate
IRIB group; regenerate Excel/PDF (128 products, version 1.1).

Co-authored-by: sharipdaitmirzaev-hue <sharipdaitmirzaev-hue@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/artifacts/commercial-price-list-2026-08-05/TINDA-Прайс-лист-финальный.xlsx
+++ b/artifacts/commercial-price-list-2026-08-05/TINDA-Прайс-лист-финальный.xlsx
@@ -10,9 +10,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Коммерческий прайс" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Коммерческий прайс'!$A$11:$L$100</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Коммерческий прайс'!$A$11:$L$150</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Коммерческий прайс'!$11:$11</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Коммерческий прайс'!$A$1:$L$100</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Коммерческий прайс'!$A$1:$L$150</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -555,7 +555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L100"/>
+  <dimension ref="A1:L150"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4.5" customWidth="1" min="1" max="1"/>
@@ -606,7 +606,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>1.1</t>
         </is>
       </c>
     </row>
@@ -4880,11 +4880,2534 @@
       <c r="K100" s="10" t="n"/>
       <c r="L100" s="9" t="n"/>
     </row>
+    <row r="101" ht="20" customHeight="1">
+      <c r="A101" s="6" t="inlineStr">
+        <is>
+          <t>IRIB</t>
+        </is>
+      </c>
+      <c r="B101" s="7" t="n"/>
+      <c r="C101" s="7" t="n"/>
+      <c r="D101" s="7" t="n"/>
+      <c r="E101" s="7" t="n"/>
+      <c r="F101" s="7" t="n"/>
+      <c r="G101" s="7" t="n"/>
+      <c r="H101" s="7" t="n"/>
+      <c r="I101" s="7" t="n"/>
+      <c r="J101" s="7" t="n"/>
+      <c r="K101" s="7" t="n"/>
+      <c r="L101" s="7" t="n"/>
+    </row>
+    <row r="102" ht="30" customHeight="1">
+      <c r="A102" s="11" t="n">
+        <v>80</v>
+      </c>
+      <c r="B102" s="12" t="inlineStr">
+        <is>
+          <t>ООО «ИРИБ»</t>
+        </is>
+      </c>
+      <c r="C102" s="12" t="inlineStr">
+        <is>
+          <t>GOLD GRAND</t>
+        </is>
+      </c>
+      <c r="D102" s="12" t="inlineStr">
+        <is>
+          <t>Лимонады</t>
+        </is>
+      </c>
+      <c r="E102" s="12" t="inlineStr">
+        <is>
+          <t>GOLD GRAND Ананас, 600 мл, ПЭТ</t>
+        </is>
+      </c>
+      <c r="F102" s="12" t="inlineStr">
+        <is>
+          <t>Ананас</t>
+        </is>
+      </c>
+      <c r="G102" s="11" t="inlineStr">
+        <is>
+          <t>600 мл</t>
+        </is>
+      </c>
+      <c r="H102" s="11" t="inlineStr">
+        <is>
+          <t>ПЭТ</t>
+        </is>
+      </c>
+      <c r="I102" s="12" t="inlineStr">
+        <is>
+          <t>IRIB-GOLD-GRAND-ANANAS-600-PET</t>
+        </is>
+      </c>
+      <c r="J102" s="12" t="inlineStr">
+        <is>
+          <t>GOLD GRAND Ананас — газированный безалкогольный напиток со вкусом «Ананас» в ПЭТ-бутылке.</t>
+        </is>
+      </c>
+      <c r="K102" s="13" t="n"/>
+      <c r="L102" s="12" t="n"/>
+    </row>
+    <row r="103" ht="45" customHeight="1">
+      <c r="A103" s="8" t="n">
+        <v>81</v>
+      </c>
+      <c r="B103" s="9" t="inlineStr">
+        <is>
+          <t>ООО «ИРИБ»</t>
+        </is>
+      </c>
+      <c r="C103" s="9" t="inlineStr">
+        <is>
+          <t>GOLD GRAND</t>
+        </is>
+      </c>
+      <c r="D103" s="9" t="inlineStr">
+        <is>
+          <t>Лимонады</t>
+        </is>
+      </c>
+      <c r="E103" s="9" t="inlineStr">
+        <is>
+          <t>GOLD GRAND Мохито негазированный, 600 мл, ПЭТ</t>
+        </is>
+      </c>
+      <c r="F103" s="9" t="inlineStr">
+        <is>
+          <t>Мохито негазированный</t>
+        </is>
+      </c>
+      <c r="G103" s="8" t="inlineStr">
+        <is>
+          <t>600 мл</t>
+        </is>
+      </c>
+      <c r="H103" s="8" t="inlineStr">
+        <is>
+          <t>ПЭТ</t>
+        </is>
+      </c>
+      <c r="I103" s="9" t="inlineStr">
+        <is>
+          <t>IRIB-GOLD-GRAND-MOHITO-NEGAZIROVANNYY-600-PET</t>
+        </is>
+      </c>
+      <c r="J103" s="9" t="inlineStr">
+        <is>
+          <t>GOLD GRAND Мохито негазированный — негазированный безалкогольный напиток со вкусом «Мохито негазированный» в ПЭТ-бутылке.</t>
+        </is>
+      </c>
+      <c r="K103" s="10" t="n"/>
+      <c r="L103" s="9" t="n"/>
+    </row>
+    <row r="104" ht="45" customHeight="1">
+      <c r="A104" s="11" t="n">
+        <v>82</v>
+      </c>
+      <c r="B104" s="12" t="inlineStr">
+        <is>
+          <t>ООО «ИРИБ»</t>
+        </is>
+      </c>
+      <c r="C104" s="12" t="inlineStr">
+        <is>
+          <t>GOLD GRAND</t>
+        </is>
+      </c>
+      <c r="D104" s="12" t="inlineStr">
+        <is>
+          <t>Лимонады</t>
+        </is>
+      </c>
+      <c r="E104" s="12" t="inlineStr">
+        <is>
+          <t>GOLD GRAND Мультифрукт, 600 мл, ПЭТ</t>
+        </is>
+      </c>
+      <c r="F104" s="12" t="inlineStr">
+        <is>
+          <t>Мультифрукт</t>
+        </is>
+      </c>
+      <c r="G104" s="11" t="inlineStr">
+        <is>
+          <t>600 мл</t>
+        </is>
+      </c>
+      <c r="H104" s="11" t="inlineStr">
+        <is>
+          <t>ПЭТ</t>
+        </is>
+      </c>
+      <c r="I104" s="12" t="inlineStr">
+        <is>
+          <t>IRIB-GOLD-GRAND-MULTIFRUKT-600-PET</t>
+        </is>
+      </c>
+      <c r="J104" s="12" t="inlineStr">
+        <is>
+          <t>GOLD GRAND Мультифрукт — газированный безалкогольный напиток со вкусом «Мультифрукт» в ПЭТ-бутылке.</t>
+        </is>
+      </c>
+      <c r="K104" s="13" t="n"/>
+      <c r="L104" s="12" t="n"/>
+    </row>
+    <row r="105" ht="30" customHeight="1">
+      <c r="A105" s="8" t="n">
+        <v>83</v>
+      </c>
+      <c r="B105" s="9" t="inlineStr">
+        <is>
+          <t>ООО «ИРИБ»</t>
+        </is>
+      </c>
+      <c r="C105" s="9" t="inlineStr">
+        <is>
+          <t>GOLD GRAND</t>
+        </is>
+      </c>
+      <c r="D105" s="9" t="inlineStr">
+        <is>
+          <t>Лимонады</t>
+        </is>
+      </c>
+      <c r="E105" s="9" t="inlineStr">
+        <is>
+          <t>GOLD GRAND Тархун, 600 мл, ПЭТ</t>
+        </is>
+      </c>
+      <c r="F105" s="9" t="inlineStr">
+        <is>
+          <t>Тархун</t>
+        </is>
+      </c>
+      <c r="G105" s="8" t="inlineStr">
+        <is>
+          <t>600 мл</t>
+        </is>
+      </c>
+      <c r="H105" s="8" t="inlineStr">
+        <is>
+          <t>ПЭТ</t>
+        </is>
+      </c>
+      <c r="I105" s="9" t="inlineStr">
+        <is>
+          <t>IRIB-GOLD-GRAND-TARHUN-600-PET</t>
+        </is>
+      </c>
+      <c r="J105" s="9" t="inlineStr">
+        <is>
+          <t>GOLD GRAND Тархун — газированный безалкогольный напиток со вкусом «Тархун» в ПЭТ-бутылке.</t>
+        </is>
+      </c>
+      <c r="K105" s="10" t="n"/>
+      <c r="L105" s="9" t="n"/>
+    </row>
+    <row r="106" ht="45" customHeight="1">
+      <c r="A106" s="11" t="n">
+        <v>84</v>
+      </c>
+      <c r="B106" s="12" t="inlineStr">
+        <is>
+          <t>ООО «ИРИБ»</t>
+        </is>
+      </c>
+      <c r="C106" s="12" t="inlineStr">
+        <is>
+          <t>Selesta</t>
+        </is>
+      </c>
+      <c r="D106" s="12" t="inlineStr">
+        <is>
+          <t>Лимонады</t>
+        </is>
+      </c>
+      <c r="E106" s="12" t="inlineStr">
+        <is>
+          <t>Selesta Ананас, 500 мл, стекло</t>
+        </is>
+      </c>
+      <c r="F106" s="12" t="inlineStr">
+        <is>
+          <t>Ананас</t>
+        </is>
+      </c>
+      <c r="G106" s="11" t="inlineStr">
+        <is>
+          <t>500 мл</t>
+        </is>
+      </c>
+      <c r="H106" s="11" t="inlineStr">
+        <is>
+          <t>стекло</t>
+        </is>
+      </c>
+      <c r="I106" s="12" t="inlineStr">
+        <is>
+          <t>IRIB-SELESTA-ANANAS-500-GLASS</t>
+        </is>
+      </c>
+      <c r="J106" s="12" t="inlineStr">
+        <is>
+          <t>Selesta Ананас — газированный безалкогольный напиток со вкусом «Ананас» в стеклянной бутылке.</t>
+        </is>
+      </c>
+      <c r="K106" s="13" t="n"/>
+      <c r="L106" s="12" t="n"/>
+    </row>
+    <row r="107" ht="45" customHeight="1">
+      <c r="A107" s="8" t="n">
+        <v>85</v>
+      </c>
+      <c r="B107" s="9" t="inlineStr">
+        <is>
+          <t>ООО «ИРИБ»</t>
+        </is>
+      </c>
+      <c r="C107" s="9" t="inlineStr">
+        <is>
+          <t>Selesta</t>
+        </is>
+      </c>
+      <c r="D107" s="9" t="inlineStr">
+        <is>
+          <t>Лимонады</t>
+        </is>
+      </c>
+      <c r="E107" s="9" t="inlineStr">
+        <is>
+          <t>Selesta Гранат, 500 мл, стекло</t>
+        </is>
+      </c>
+      <c r="F107" s="9" t="inlineStr">
+        <is>
+          <t>Гранат</t>
+        </is>
+      </c>
+      <c r="G107" s="8" t="inlineStr">
+        <is>
+          <t>500 мл</t>
+        </is>
+      </c>
+      <c r="H107" s="8" t="inlineStr">
+        <is>
+          <t>стекло</t>
+        </is>
+      </c>
+      <c r="I107" s="9" t="inlineStr">
+        <is>
+          <t>IRIB-SELESTA-GRANAT-500-GLASS</t>
+        </is>
+      </c>
+      <c r="J107" s="9" t="inlineStr">
+        <is>
+          <t>Selesta Гранат — газированный безалкогольный напиток со вкусом «Гранат» в стеклянной бутылке.</t>
+        </is>
+      </c>
+      <c r="K107" s="10" t="n"/>
+      <c r="L107" s="9" t="n"/>
+    </row>
+    <row r="108" ht="45" customHeight="1">
+      <c r="A108" s="11" t="n">
+        <v>86</v>
+      </c>
+      <c r="B108" s="12" t="inlineStr">
+        <is>
+          <t>ООО «ИРИБ»</t>
+        </is>
+      </c>
+      <c r="C108" s="12" t="inlineStr">
+        <is>
+          <t>Selesta</t>
+        </is>
+      </c>
+      <c r="D108" s="12" t="inlineStr">
+        <is>
+          <t>Лимонады</t>
+        </is>
+      </c>
+      <c r="E108" s="12" t="inlineStr">
+        <is>
+          <t>Selesta Груша, 500 мл, стекло</t>
+        </is>
+      </c>
+      <c r="F108" s="12" t="inlineStr">
+        <is>
+          <t>Груша</t>
+        </is>
+      </c>
+      <c r="G108" s="11" t="inlineStr">
+        <is>
+          <t>500 мл</t>
+        </is>
+      </c>
+      <c r="H108" s="11" t="inlineStr">
+        <is>
+          <t>стекло</t>
+        </is>
+      </c>
+      <c r="I108" s="12" t="inlineStr">
+        <is>
+          <t>IRIB-SELESTA-GRUSHA-500-GLASS</t>
+        </is>
+      </c>
+      <c r="J108" s="12" t="inlineStr">
+        <is>
+          <t>Selesta Груша — газированный безалкогольный напиток со вкусом «Груша» в стеклянной бутылке.</t>
+        </is>
+      </c>
+      <c r="K108" s="13" t="n"/>
+      <c r="L108" s="12" t="n"/>
+    </row>
+    <row r="109" ht="45" customHeight="1">
+      <c r="A109" s="8" t="n">
+        <v>87</v>
+      </c>
+      <c r="B109" s="9" t="inlineStr">
+        <is>
+          <t>ООО «ИРИБ»</t>
+        </is>
+      </c>
+      <c r="C109" s="9" t="inlineStr">
+        <is>
+          <t>Selesta</t>
+        </is>
+      </c>
+      <c r="D109" s="9" t="inlineStr">
+        <is>
+          <t>Лимонады</t>
+        </is>
+      </c>
+      <c r="E109" s="9" t="inlineStr">
+        <is>
+          <t>Selesta Мохито, 500 мл, стекло</t>
+        </is>
+      </c>
+      <c r="F109" s="9" t="inlineStr">
+        <is>
+          <t>Мохито</t>
+        </is>
+      </c>
+      <c r="G109" s="8" t="inlineStr">
+        <is>
+          <t>500 мл</t>
+        </is>
+      </c>
+      <c r="H109" s="8" t="inlineStr">
+        <is>
+          <t>стекло</t>
+        </is>
+      </c>
+      <c r="I109" s="9" t="inlineStr">
+        <is>
+          <t>IRIB-SELESTA-MOHITO-500-GLASS</t>
+        </is>
+      </c>
+      <c r="J109" s="9" t="inlineStr">
+        <is>
+          <t>Selesta Мохито — газированный безалкогольный напиток со вкусом «Мохито» в стеклянной бутылке.</t>
+        </is>
+      </c>
+      <c r="K109" s="10" t="n"/>
+      <c r="L109" s="9" t="n"/>
+    </row>
+    <row r="110" ht="45" customHeight="1">
+      <c r="A110" s="11" t="n">
+        <v>88</v>
+      </c>
+      <c r="B110" s="12" t="inlineStr">
+        <is>
+          <t>ООО «ИРИБ»</t>
+        </is>
+      </c>
+      <c r="C110" s="12" t="inlineStr">
+        <is>
+          <t>Selesta</t>
+        </is>
+      </c>
+      <c r="D110" s="12" t="inlineStr">
+        <is>
+          <t>Лимонады</t>
+        </is>
+      </c>
+      <c r="E110" s="12" t="inlineStr">
+        <is>
+          <t>Selesta Мультифрукт, 750 мл, стекло</t>
+        </is>
+      </c>
+      <c r="F110" s="12" t="inlineStr">
+        <is>
+          <t>Мультифрукт</t>
+        </is>
+      </c>
+      <c r="G110" s="11" t="inlineStr">
+        <is>
+          <t>750 мл</t>
+        </is>
+      </c>
+      <c r="H110" s="11" t="inlineStr">
+        <is>
+          <t>стекло</t>
+        </is>
+      </c>
+      <c r="I110" s="12" t="inlineStr">
+        <is>
+          <t>IRIB-SELESTA-MULTIFRUKT-750-GLASS</t>
+        </is>
+      </c>
+      <c r="J110" s="12" t="inlineStr">
+        <is>
+          <t>Selesta Мультифрукт — газированный безалкогольный напиток со вкусом «Мультифрукт» в стеклянной бутылке.</t>
+        </is>
+      </c>
+      <c r="K110" s="13" t="n"/>
+      <c r="L110" s="12" t="n"/>
+    </row>
+    <row r="111" ht="45" customHeight="1">
+      <c r="A111" s="8" t="n">
+        <v>89</v>
+      </c>
+      <c r="B111" s="9" t="inlineStr">
+        <is>
+          <t>ООО «ИРИБ»</t>
+        </is>
+      </c>
+      <c r="C111" s="9" t="inlineStr">
+        <is>
+          <t>Selesta</t>
+        </is>
+      </c>
+      <c r="D111" s="9" t="inlineStr">
+        <is>
+          <t>Лимонады</t>
+        </is>
+      </c>
+      <c r="E111" s="9" t="inlineStr">
+        <is>
+          <t>Selesta Шиповник, 500 мл, стекло</t>
+        </is>
+      </c>
+      <c r="F111" s="9" t="inlineStr">
+        <is>
+          <t>Шиповник</t>
+        </is>
+      </c>
+      <c r="G111" s="8" t="inlineStr">
+        <is>
+          <t>500 мл</t>
+        </is>
+      </c>
+      <c r="H111" s="8" t="inlineStr">
+        <is>
+          <t>стекло</t>
+        </is>
+      </c>
+      <c r="I111" s="9" t="inlineStr">
+        <is>
+          <t>IRIB-SELESTA-SHIPOVNIK-500-GLASS</t>
+        </is>
+      </c>
+      <c r="J111" s="9" t="inlineStr">
+        <is>
+          <t>Selesta Шиповник — газированный безалкогольный напиток со вкусом «Шиповник» в стеклянной бутылке.</t>
+        </is>
+      </c>
+      <c r="K111" s="10" t="n"/>
+      <c r="L111" s="9" t="n"/>
+    </row>
+    <row r="112" ht="45" customHeight="1">
+      <c r="A112" s="11" t="n">
+        <v>90</v>
+      </c>
+      <c r="B112" s="12" t="inlineStr">
+        <is>
+          <t>ООО «ИРИБ»</t>
+        </is>
+      </c>
+      <c r="C112" s="12" t="inlineStr">
+        <is>
+          <t>Талих</t>
+        </is>
+      </c>
+      <c r="D112" s="12" t="inlineStr">
+        <is>
+          <t>Газированные напитки</t>
+        </is>
+      </c>
+      <c r="E112" s="12" t="inlineStr">
+        <is>
+          <t>Талих Классический, 600 мл, ПЭТ</t>
+        </is>
+      </c>
+      <c r="F112" s="12" t="inlineStr">
+        <is>
+          <t>Классический</t>
+        </is>
+      </c>
+      <c r="G112" s="11" t="inlineStr">
+        <is>
+          <t>600 мл</t>
+        </is>
+      </c>
+      <c r="H112" s="11" t="inlineStr">
+        <is>
+          <t>ПЭТ</t>
+        </is>
+      </c>
+      <c r="I112" s="12" t="inlineStr">
+        <is>
+          <t>IRIB-TALIH-SPORT-KLASSICHESKIY-600-PET</t>
+        </is>
+      </c>
+      <c r="J112" s="12" t="inlineStr">
+        <is>
+          <t>Талих Классический — газированный безалкогольный напиток со вкусом «Классический» в ПЭТ-бутылке.</t>
+        </is>
+      </c>
+      <c r="K112" s="13" t="n"/>
+      <c r="L112" s="12" t="n"/>
+    </row>
+    <row r="113" ht="30" customHeight="1">
+      <c r="A113" s="8" t="n">
+        <v>91</v>
+      </c>
+      <c r="B113" s="9" t="inlineStr">
+        <is>
+          <t>ООО «ИРИБ»</t>
+        </is>
+      </c>
+      <c r="C113" s="9" t="inlineStr">
+        <is>
+          <t>Талих</t>
+        </is>
+      </c>
+      <c r="D113" s="9" t="inlineStr">
+        <is>
+          <t>Газированные напитки</t>
+        </is>
+      </c>
+      <c r="E113" s="9" t="inlineStr">
+        <is>
+          <t>Талих Клубника, 600 мл, ПЭТ</t>
+        </is>
+      </c>
+      <c r="F113" s="9" t="inlineStr">
+        <is>
+          <t>Клубника</t>
+        </is>
+      </c>
+      <c r="G113" s="8" t="inlineStr">
+        <is>
+          <t>600 мл</t>
+        </is>
+      </c>
+      <c r="H113" s="8" t="inlineStr">
+        <is>
+          <t>ПЭТ</t>
+        </is>
+      </c>
+      <c r="I113" s="9" t="inlineStr">
+        <is>
+          <t>IRIB-TALIH-SPORT-KLUBNIKA-600-PET</t>
+        </is>
+      </c>
+      <c r="J113" s="9" t="inlineStr">
+        <is>
+          <t>Талих Клубника — газированный безалкогольный напиток со вкусом «Клубника» в ПЭТ-бутылке.</t>
+        </is>
+      </c>
+      <c r="K113" s="10" t="n"/>
+      <c r="L113" s="9" t="n"/>
+    </row>
+    <row r="114" ht="30" customHeight="1">
+      <c r="A114" s="11" t="n">
+        <v>92</v>
+      </c>
+      <c r="B114" s="12" t="inlineStr">
+        <is>
+          <t>ООО «ИРИБ»</t>
+        </is>
+      </c>
+      <c r="C114" s="12" t="inlineStr">
+        <is>
+          <t>Талих</t>
+        </is>
+      </c>
+      <c r="D114" s="12" t="inlineStr">
+        <is>
+          <t>Газированные напитки</t>
+        </is>
+      </c>
+      <c r="E114" s="12" t="inlineStr">
+        <is>
+          <t>Талих Лимон, 600 мл, ПЭТ</t>
+        </is>
+      </c>
+      <c r="F114" s="12" t="inlineStr">
+        <is>
+          <t>Лимон</t>
+        </is>
+      </c>
+      <c r="G114" s="11" t="inlineStr">
+        <is>
+          <t>600 мл</t>
+        </is>
+      </c>
+      <c r="H114" s="11" t="inlineStr">
+        <is>
+          <t>ПЭТ</t>
+        </is>
+      </c>
+      <c r="I114" s="12" t="inlineStr">
+        <is>
+          <t>IRIB-TALIH-SPORT-LIMON-600-PET</t>
+        </is>
+      </c>
+      <c r="J114" s="12" t="inlineStr">
+        <is>
+          <t>Талих Лимон — газированный безалкогольный напиток со вкусом «Лимон» в ПЭТ-бутылке.</t>
+        </is>
+      </c>
+      <c r="K114" s="13" t="n"/>
+      <c r="L114" s="12" t="n"/>
+    </row>
+    <row r="115" ht="30" customHeight="1">
+      <c r="A115" s="8" t="n">
+        <v>93</v>
+      </c>
+      <c r="B115" s="9" t="inlineStr">
+        <is>
+          <t>ООО «ИРИБ»</t>
+        </is>
+      </c>
+      <c r="C115" s="9" t="inlineStr">
+        <is>
+          <t>Ice Bar</t>
+        </is>
+      </c>
+      <c r="D115" s="9" t="inlineStr">
+        <is>
+          <t>Холодный чай</t>
+        </is>
+      </c>
+      <c r="E115" s="9" t="inlineStr">
+        <is>
+          <t>Ice Bar манго-клубника, 500 мл, ПЭТ</t>
+        </is>
+      </c>
+      <c r="F115" s="9" t="inlineStr">
+        <is>
+          <t>манго-клубника</t>
+        </is>
+      </c>
+      <c r="G115" s="8" t="inlineStr">
+        <is>
+          <t>500 мл</t>
+        </is>
+      </c>
+      <c r="H115" s="8" t="inlineStr">
+        <is>
+          <t>ПЭТ</t>
+        </is>
+      </c>
+      <c r="I115" s="9" t="inlineStr">
+        <is>
+          <t>IRIB-ICE-BAR-MANGO-KLUBNIKA-500-PET</t>
+        </is>
+      </c>
+      <c r="J115" s="9" t="inlineStr">
+        <is>
+          <t>Ice Bar манго-клубника — холодный чай со вкусом «манго-клубника» в ПЭТ-бутылке.</t>
+        </is>
+      </c>
+      <c r="K115" s="10" t="n"/>
+      <c r="L115" s="9" t="n"/>
+    </row>
+    <row r="116" ht="30" customHeight="1">
+      <c r="A116" s="11" t="n">
+        <v>94</v>
+      </c>
+      <c r="B116" s="12" t="inlineStr">
+        <is>
+          <t>ООО «ИРИБ»</t>
+        </is>
+      </c>
+      <c r="C116" s="12" t="inlineStr">
+        <is>
+          <t>Ice Bar</t>
+        </is>
+      </c>
+      <c r="D116" s="12" t="inlineStr">
+        <is>
+          <t>Холодный чай</t>
+        </is>
+      </c>
+      <c r="E116" s="12" t="inlineStr">
+        <is>
+          <t>Ice Bar Персик, 500 мл, ПЭТ</t>
+        </is>
+      </c>
+      <c r="F116" s="12" t="inlineStr">
+        <is>
+          <t>Персик</t>
+        </is>
+      </c>
+      <c r="G116" s="11" t="inlineStr">
+        <is>
+          <t>500 мл</t>
+        </is>
+      </c>
+      <c r="H116" s="11" t="inlineStr">
+        <is>
+          <t>ПЭТ</t>
+        </is>
+      </c>
+      <c r="I116" s="12" t="inlineStr">
+        <is>
+          <t>IRIB-ICE-BAR-PERSIK-500-PET</t>
+        </is>
+      </c>
+      <c r="J116" s="12" t="inlineStr">
+        <is>
+          <t>Ice Bar Персик — холодный чай со вкусом «Персик» в ПЭТ-бутылке.</t>
+        </is>
+      </c>
+      <c r="K116" s="13" t="n"/>
+      <c r="L116" s="12" t="n"/>
+    </row>
+    <row r="117" ht="30" customHeight="1">
+      <c r="A117" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="B117" s="9" t="inlineStr">
+        <is>
+          <t>ООО «ИРИБ»</t>
+        </is>
+      </c>
+      <c r="C117" s="9" t="inlineStr">
+        <is>
+          <t>Ice Bar</t>
+        </is>
+      </c>
+      <c r="D117" s="9" t="inlineStr">
+        <is>
+          <t>Холодный чай</t>
+        </is>
+      </c>
+      <c r="E117" s="9" t="inlineStr">
+        <is>
+          <t>Ice Bar Ягодный, 500 мл, ПЭТ</t>
+        </is>
+      </c>
+      <c r="F117" s="9" t="inlineStr">
+        <is>
+          <t>Ягодный</t>
+        </is>
+      </c>
+      <c r="G117" s="8" t="inlineStr">
+        <is>
+          <t>500 мл</t>
+        </is>
+      </c>
+      <c r="H117" s="8" t="inlineStr">
+        <is>
+          <t>ПЭТ</t>
+        </is>
+      </c>
+      <c r="I117" s="9" t="inlineStr">
+        <is>
+          <t>IRIB-ICE-BAR-YAGODNYY-500-PET</t>
+        </is>
+      </c>
+      <c r="J117" s="9" t="inlineStr">
+        <is>
+          <t>Ice Bar Ягодный — холодный чай со вкусом «Ягодный» в ПЭТ-бутылке.</t>
+        </is>
+      </c>
+      <c r="K117" s="10" t="n"/>
+      <c r="L117" s="9" t="n"/>
+    </row>
+    <row r="118" ht="30" customHeight="1">
+      <c r="A118" s="11" t="n">
+        <v>96</v>
+      </c>
+      <c r="B118" s="12" t="inlineStr">
+        <is>
+          <t>ООО «ИРИБ»</t>
+        </is>
+      </c>
+      <c r="C118" s="12" t="inlineStr">
+        <is>
+          <t>Ириб</t>
+        </is>
+      </c>
+      <c r="D118" s="12" t="inlineStr">
+        <is>
+          <t>Квас</t>
+        </is>
+      </c>
+      <c r="E118" s="12" t="inlineStr">
+        <is>
+          <t>Квас Ириб Янтарный, 1,25 л, ПЭТ</t>
+        </is>
+      </c>
+      <c r="F118" s="12" t="inlineStr">
+        <is>
+          <t>Янтарный</t>
+        </is>
+      </c>
+      <c r="G118" s="11" t="inlineStr">
+        <is>
+          <t>1,25 л</t>
+        </is>
+      </c>
+      <c r="H118" s="11" t="inlineStr">
+        <is>
+          <t>ПЭТ</t>
+        </is>
+      </c>
+      <c r="I118" s="12" t="inlineStr">
+        <is>
+          <t>IRIB-KVAS-YANTARNYY-1250-PET</t>
+        </is>
+      </c>
+      <c r="J118" s="12" t="inlineStr">
+        <is>
+          <t>Ириб Янтарный — квас в ПЭТ-бутылке.</t>
+        </is>
+      </c>
+      <c r="K118" s="13" t="n"/>
+      <c r="L118" s="12" t="n"/>
+    </row>
+    <row r="119" ht="30" customHeight="1">
+      <c r="A119" s="8" t="n">
+        <v>97</v>
+      </c>
+      <c r="B119" s="9" t="inlineStr">
+        <is>
+          <t>ООО «ИРИБ»</t>
+        </is>
+      </c>
+      <c r="C119" s="9" t="inlineStr">
+        <is>
+          <t>PROFI SPORT</t>
+        </is>
+      </c>
+      <c r="D119" s="9" t="inlineStr">
+        <is>
+          <t>Энергетические напитки</t>
+        </is>
+      </c>
+      <c r="E119" s="9" t="inlineStr">
+        <is>
+          <t>PROFI SPORT Energy Гуарана, 500 мл, ПЭТ</t>
+        </is>
+      </c>
+      <c r="F119" s="9" t="inlineStr">
+        <is>
+          <t>Energy Гуарана</t>
+        </is>
+      </c>
+      <c r="G119" s="8" t="inlineStr">
+        <is>
+          <t>500 мл</t>
+        </is>
+      </c>
+      <c r="H119" s="8" t="inlineStr">
+        <is>
+          <t>ПЭТ</t>
+        </is>
+      </c>
+      <c r="I119" s="9" t="inlineStr">
+        <is>
+          <t>IRIB-PROFI-SPORT-ENERGY-GUARANA-500-PET</t>
+        </is>
+      </c>
+      <c r="J119" s="9" t="inlineStr">
+        <is>
+          <t>PROFI SPORT Energy Гуарана — безалкогольный энергетический напиток в ПЭТ-бутылке.</t>
+        </is>
+      </c>
+      <c r="K119" s="10" t="n"/>
+      <c r="L119" s="9" t="n"/>
+    </row>
+    <row r="120" ht="30" customHeight="1">
+      <c r="A120" s="11" t="n">
+        <v>98</v>
+      </c>
+      <c r="B120" s="12" t="inlineStr">
+        <is>
+          <t>ООО «ИРИБ»</t>
+        </is>
+      </c>
+      <c r="C120" s="12" t="inlineStr">
+        <is>
+          <t>Ириб</t>
+        </is>
+      </c>
+      <c r="D120" s="12" t="inlineStr">
+        <is>
+          <t>Сок</t>
+        </is>
+      </c>
+      <c r="E120" s="12" t="inlineStr">
+        <is>
+          <t>Сок Ириб Ананасовый, 500 мл, стекло</t>
+        </is>
+      </c>
+      <c r="F120" s="12" t="inlineStr">
+        <is>
+          <t>Ананасовый</t>
+        </is>
+      </c>
+      <c r="G120" s="11" t="inlineStr">
+        <is>
+          <t>500 мл</t>
+        </is>
+      </c>
+      <c r="H120" s="11" t="inlineStr">
+        <is>
+          <t>стекло</t>
+        </is>
+      </c>
+      <c r="I120" s="12" t="inlineStr">
+        <is>
+          <t>IRIB-SOK-ANANASOVYY-500-GLASS</t>
+        </is>
+      </c>
+      <c r="J120" s="12" t="inlineStr">
+        <is>
+          <t>Ириб Ананасовый — фруктовый сок в стеклянной бутылке.</t>
+        </is>
+      </c>
+      <c r="K120" s="13" t="n"/>
+      <c r="L120" s="12" t="n"/>
+    </row>
+    <row r="121" ht="30" customHeight="1">
+      <c r="A121" s="8" t="n">
+        <v>99</v>
+      </c>
+      <c r="B121" s="9" t="inlineStr">
+        <is>
+          <t>ООО «ИРИБ»</t>
+        </is>
+      </c>
+      <c r="C121" s="9" t="inlineStr">
+        <is>
+          <t>Ириб</t>
+        </is>
+      </c>
+      <c r="D121" s="9" t="inlineStr">
+        <is>
+          <t>Сок</t>
+        </is>
+      </c>
+      <c r="E121" s="9" t="inlineStr">
+        <is>
+          <t>Сок Ириб Мультифруктовый, 750 мл, стекло</t>
+        </is>
+      </c>
+      <c r="F121" s="9" t="inlineStr">
+        <is>
+          <t>Мультифруктовый</t>
+        </is>
+      </c>
+      <c r="G121" s="8" t="inlineStr">
+        <is>
+          <t>750 мл</t>
+        </is>
+      </c>
+      <c r="H121" s="8" t="inlineStr">
+        <is>
+          <t>стекло</t>
+        </is>
+      </c>
+      <c r="I121" s="9" t="inlineStr">
+        <is>
+          <t>IRIB-SOK-MULTIFRUKTOVYY-750-GLASS</t>
+        </is>
+      </c>
+      <c r="J121" s="9" t="inlineStr">
+        <is>
+          <t>Ириб Мультифруктовый — фруктовый сок в стеклянной бутылке.</t>
+        </is>
+      </c>
+      <c r="K121" s="10" t="n"/>
+      <c r="L121" s="9" t="n"/>
+    </row>
+    <row r="122" ht="30" customHeight="1">
+      <c r="A122" s="11" t="n">
+        <v>100</v>
+      </c>
+      <c r="B122" s="12" t="inlineStr">
+        <is>
+          <t>ООО «ИРИБ»</t>
+        </is>
+      </c>
+      <c r="C122" s="12" t="inlineStr">
+        <is>
+          <t>Ириб</t>
+        </is>
+      </c>
+      <c r="D122" s="12" t="inlineStr">
+        <is>
+          <t>Сок</t>
+        </is>
+      </c>
+      <c r="E122" s="12" t="inlineStr">
+        <is>
+          <t>Сок Ириб Яблочный, 500 мл, стекло</t>
+        </is>
+      </c>
+      <c r="F122" s="12" t="inlineStr">
+        <is>
+          <t>Яблочный</t>
+        </is>
+      </c>
+      <c r="G122" s="11" t="inlineStr">
+        <is>
+          <t>500 мл</t>
+        </is>
+      </c>
+      <c r="H122" s="11" t="inlineStr">
+        <is>
+          <t>стекло</t>
+        </is>
+      </c>
+      <c r="I122" s="12" t="inlineStr">
+        <is>
+          <t>IRIB-SOK-YABLOCHNYY-500-GLASS</t>
+        </is>
+      </c>
+      <c r="J122" s="12" t="inlineStr">
+        <is>
+          <t>Ириб Яблочный — фруктовый сок в стеклянной бутылке.</t>
+        </is>
+      </c>
+      <c r="K122" s="13" t="n"/>
+      <c r="L122" s="12" t="n"/>
+    </row>
+    <row r="123" ht="30" customHeight="1">
+      <c r="A123" s="8" t="n">
+        <v>101</v>
+      </c>
+      <c r="B123" s="9" t="inlineStr">
+        <is>
+          <t>ООО «ИРИБ»</t>
+        </is>
+      </c>
+      <c r="C123" s="9" t="inlineStr">
+        <is>
+          <t>Ириб</t>
+        </is>
+      </c>
+      <c r="D123" s="9" t="inlineStr">
+        <is>
+          <t>Сок</t>
+        </is>
+      </c>
+      <c r="E123" s="9" t="inlineStr">
+        <is>
+          <t>Сок Ириб Яблочный, 3 л, ПЭТ</t>
+        </is>
+      </c>
+      <c r="F123" s="9" t="inlineStr">
+        <is>
+          <t>Яблочный</t>
+        </is>
+      </c>
+      <c r="G123" s="8" t="inlineStr">
+        <is>
+          <t>3 л</t>
+        </is>
+      </c>
+      <c r="H123" s="8" t="inlineStr">
+        <is>
+          <t>ПЭТ</t>
+        </is>
+      </c>
+      <c r="I123" s="9" t="inlineStr">
+        <is>
+          <t>IRIB-SOK-YABLOCHNYY-3000-PET</t>
+        </is>
+      </c>
+      <c r="J123" s="9" t="inlineStr">
+        <is>
+          <t>Ириб Яблочный — фруктовый сок в ПЭТ-бутылке.</t>
+        </is>
+      </c>
+      <c r="K123" s="10" t="n"/>
+      <c r="L123" s="9" t="n"/>
+    </row>
+    <row r="124" ht="30" customHeight="1">
+      <c r="A124" s="11" t="n">
+        <v>102</v>
+      </c>
+      <c r="B124" s="12" t="inlineStr"/>
+      <c r="C124" s="12" t="inlineStr">
+        <is>
+          <t>Ириб</t>
+        </is>
+      </c>
+      <c r="D124" s="12" t="inlineStr">
+        <is>
+          <t>Сок</t>
+        </is>
+      </c>
+      <c r="E124" s="12" t="inlineStr">
+        <is>
+          <t>Сок Ириб ст/б 0,75л Ананасовый 100%</t>
+        </is>
+      </c>
+      <c r="F124" s="12" t="inlineStr">
+        <is>
+          <t>Ананасовый</t>
+        </is>
+      </c>
+      <c r="G124" s="11" t="inlineStr">
+        <is>
+          <t>750 мл</t>
+        </is>
+      </c>
+      <c r="H124" s="11" t="inlineStr">
+        <is>
+          <t>стекло</t>
+        </is>
+      </c>
+      <c r="I124" s="12" t="inlineStr">
+        <is>
+          <t>ZY-IRIB-750-GLASS-009</t>
+        </is>
+      </c>
+      <c r="J124" s="12" t="inlineStr">
+        <is>
+          <t>Ириб Ананасовый — фруктовый сок в стеклянной бутылке.</t>
+        </is>
+      </c>
+      <c r="K124" s="13" t="n"/>
+      <c r="L124" s="12" t="n"/>
+    </row>
+    <row r="125" ht="30" customHeight="1">
+      <c r="A125" s="8" t="n">
+        <v>103</v>
+      </c>
+      <c r="B125" s="9" t="inlineStr"/>
+      <c r="C125" s="9" t="inlineStr">
+        <is>
+          <t>Ириб</t>
+        </is>
+      </c>
+      <c r="D125" s="9" t="inlineStr">
+        <is>
+          <t>Сок</t>
+        </is>
+      </c>
+      <c r="E125" s="9" t="inlineStr">
+        <is>
+          <t>Сок Ириб ст/б 0,75л Апельсиновый 100%</t>
+        </is>
+      </c>
+      <c r="F125" s="9" t="inlineStr">
+        <is>
+          <t>Апельсиновый</t>
+        </is>
+      </c>
+      <c r="G125" s="8" t="inlineStr">
+        <is>
+          <t>750 мл</t>
+        </is>
+      </c>
+      <c r="H125" s="8" t="inlineStr">
+        <is>
+          <t>стекло</t>
+        </is>
+      </c>
+      <c r="I125" s="9" t="inlineStr">
+        <is>
+          <t>ZY-IRIB-750-GLASS-007</t>
+        </is>
+      </c>
+      <c r="J125" s="9" t="inlineStr">
+        <is>
+          <t>Ириб Апельсиновый — фруктовый сок в стеклянной бутылке.</t>
+        </is>
+      </c>
+      <c r="K125" s="10" t="n"/>
+      <c r="L125" s="9" t="n"/>
+    </row>
+    <row r="126" ht="30" customHeight="1">
+      <c r="A126" s="11" t="n">
+        <v>104</v>
+      </c>
+      <c r="B126" s="12" t="inlineStr"/>
+      <c r="C126" s="12" t="inlineStr">
+        <is>
+          <t>Ириб</t>
+        </is>
+      </c>
+      <c r="D126" s="12" t="inlineStr">
+        <is>
+          <t>Сок</t>
+        </is>
+      </c>
+      <c r="E126" s="12" t="inlineStr">
+        <is>
+          <t>Сок Ириб ст/б 0,75л виноградный красный 100%</t>
+        </is>
+      </c>
+      <c r="F126" s="12" t="inlineStr">
+        <is>
+          <t>виноградный красный</t>
+        </is>
+      </c>
+      <c r="G126" s="11" t="inlineStr">
+        <is>
+          <t>750 мл</t>
+        </is>
+      </c>
+      <c r="H126" s="11" t="inlineStr">
+        <is>
+          <t>стекло</t>
+        </is>
+      </c>
+      <c r="I126" s="12" t="inlineStr">
+        <is>
+          <t>ZY-IRIB-750-GLASS-008</t>
+        </is>
+      </c>
+      <c r="J126" s="12" t="inlineStr">
+        <is>
+          <t>Ириб виноградный красный — фруктовый сок в стеклянной бутылке.</t>
+        </is>
+      </c>
+      <c r="K126" s="13" t="n"/>
+      <c r="L126" s="12" t="n"/>
+    </row>
+    <row r="127" ht="30" customHeight="1">
+      <c r="A127" s="8" t="n">
+        <v>105</v>
+      </c>
+      <c r="B127" s="9" t="inlineStr"/>
+      <c r="C127" s="9" t="inlineStr">
+        <is>
+          <t>Ириб</t>
+        </is>
+      </c>
+      <c r="D127" s="9" t="inlineStr">
+        <is>
+          <t>Сок</t>
+        </is>
+      </c>
+      <c r="E127" s="9" t="inlineStr">
+        <is>
+          <t>Сок Ириб ст/б 0,75л Гранатовый 100%</t>
+        </is>
+      </c>
+      <c r="F127" s="9" t="inlineStr">
+        <is>
+          <t>Гранатовый</t>
+        </is>
+      </c>
+      <c r="G127" s="8" t="inlineStr">
+        <is>
+          <t>750 мл</t>
+        </is>
+      </c>
+      <c r="H127" s="8" t="inlineStr">
+        <is>
+          <t>стекло</t>
+        </is>
+      </c>
+      <c r="I127" s="9" t="inlineStr">
+        <is>
+          <t>ZY-IRIB-750-GLASS-001</t>
+        </is>
+      </c>
+      <c r="J127" s="9" t="inlineStr">
+        <is>
+          <t>Ириб Гранатовый — фруктовый сок в стеклянной бутылке.</t>
+        </is>
+      </c>
+      <c r="K127" s="10" t="n"/>
+      <c r="L127" s="9" t="n"/>
+    </row>
+    <row r="128" ht="30" customHeight="1">
+      <c r="A128" s="11" t="n">
+        <v>106</v>
+      </c>
+      <c r="B128" s="12" t="inlineStr"/>
+      <c r="C128" s="12" t="inlineStr">
+        <is>
+          <t>Ириб</t>
+        </is>
+      </c>
+      <c r="D128" s="12" t="inlineStr">
+        <is>
+          <t>Сок</t>
+        </is>
+      </c>
+      <c r="E128" s="12" t="inlineStr">
+        <is>
+          <t>Сок Ириб ст/б 0,75л Томатный 100%</t>
+        </is>
+      </c>
+      <c r="F128" s="12" t="inlineStr">
+        <is>
+          <t>Томатный</t>
+        </is>
+      </c>
+      <c r="G128" s="11" t="inlineStr">
+        <is>
+          <t>750 мл</t>
+        </is>
+      </c>
+      <c r="H128" s="11" t="inlineStr">
+        <is>
+          <t>стекло</t>
+        </is>
+      </c>
+      <c r="I128" s="12" t="inlineStr">
+        <is>
+          <t>ZY-IRIB-750-GLASS-011</t>
+        </is>
+      </c>
+      <c r="J128" s="12" t="inlineStr">
+        <is>
+          <t>Ириб Томатный — фруктовый сок в стеклянной бутылке.</t>
+        </is>
+      </c>
+      <c r="K128" s="13" t="n"/>
+      <c r="L128" s="12" t="n"/>
+    </row>
+    <row r="129" ht="30" customHeight="1">
+      <c r="A129" s="8" t="n">
+        <v>107</v>
+      </c>
+      <c r="B129" s="9" t="inlineStr"/>
+      <c r="C129" s="9" t="inlineStr">
+        <is>
+          <t>Ириб</t>
+        </is>
+      </c>
+      <c r="D129" s="9" t="inlineStr">
+        <is>
+          <t>Сок</t>
+        </is>
+      </c>
+      <c r="E129" s="9" t="inlineStr">
+        <is>
+          <t>Сок Ириб ст/б 0,33л Яблочный 100%</t>
+        </is>
+      </c>
+      <c r="F129" s="9" t="inlineStr">
+        <is>
+          <t>Яблочный</t>
+        </is>
+      </c>
+      <c r="G129" s="8" t="inlineStr">
+        <is>
+          <t>330 мл</t>
+        </is>
+      </c>
+      <c r="H129" s="8" t="inlineStr">
+        <is>
+          <t>стекло</t>
+        </is>
+      </c>
+      <c r="I129" s="9" t="inlineStr">
+        <is>
+          <t>ZY-IRIB-330-GLASS-001</t>
+        </is>
+      </c>
+      <c r="J129" s="9" t="inlineStr">
+        <is>
+          <t>Ириб Яблочный — фруктовый сок в стеклянной бутылке.</t>
+        </is>
+      </c>
+      <c r="K129" s="10" t="n"/>
+      <c r="L129" s="9" t="n"/>
+    </row>
+    <row r="130" ht="30" customHeight="1">
+      <c r="A130" s="11" t="n">
+        <v>108</v>
+      </c>
+      <c r="B130" s="12" t="inlineStr"/>
+      <c r="C130" s="12" t="inlineStr">
+        <is>
+          <t>Ириб</t>
+        </is>
+      </c>
+      <c r="D130" s="12" t="inlineStr">
+        <is>
+          <t>Сок</t>
+        </is>
+      </c>
+      <c r="E130" s="12" t="inlineStr">
+        <is>
+          <t>Сок Ириб ст/б 0,75л Яблочный 100%</t>
+        </is>
+      </c>
+      <c r="F130" s="12" t="inlineStr">
+        <is>
+          <t>Яблочный</t>
+        </is>
+      </c>
+      <c r="G130" s="11" t="inlineStr">
+        <is>
+          <t>750 мл</t>
+        </is>
+      </c>
+      <c r="H130" s="11" t="inlineStr">
+        <is>
+          <t>стекло</t>
+        </is>
+      </c>
+      <c r="I130" s="12" t="inlineStr">
+        <is>
+          <t>ZY-IRIB-750-GLASS-005</t>
+        </is>
+      </c>
+      <c r="J130" s="12" t="inlineStr">
+        <is>
+          <t>Ириб Яблочный — фруктовый сок в стеклянной бутылке.</t>
+        </is>
+      </c>
+      <c r="K130" s="13" t="n"/>
+      <c r="L130" s="12" t="n"/>
+    </row>
+    <row r="131" ht="30" customHeight="1">
+      <c r="A131" s="8" t="n">
+        <v>109</v>
+      </c>
+      <c r="B131" s="9" t="inlineStr">
+        <is>
+          <t>ООО «ИРИБ»</t>
+        </is>
+      </c>
+      <c r="C131" s="9" t="inlineStr">
+        <is>
+          <t>Ириб</t>
+        </is>
+      </c>
+      <c r="D131" s="9" t="inlineStr">
+        <is>
+          <t>Нектар</t>
+        </is>
+      </c>
+      <c r="E131" s="9" t="inlineStr">
+        <is>
+          <t>Нектар Ириб Абрикосовый, 500 мл, стекло</t>
+        </is>
+      </c>
+      <c r="F131" s="9" t="inlineStr">
+        <is>
+          <t>Абрикосовый</t>
+        </is>
+      </c>
+      <c r="G131" s="8" t="inlineStr">
+        <is>
+          <t>500 мл</t>
+        </is>
+      </c>
+      <c r="H131" s="8" t="inlineStr">
+        <is>
+          <t>стекло</t>
+        </is>
+      </c>
+      <c r="I131" s="9" t="inlineStr">
+        <is>
+          <t>IRIB-NEKTAR-ABRIKOSOVYY-500-GLASS</t>
+        </is>
+      </c>
+      <c r="J131" s="9" t="inlineStr">
+        <is>
+          <t>Ириб Абрикосовый — фруктовый нектар в стеклянной бутылке.</t>
+        </is>
+      </c>
+      <c r="K131" s="10" t="n"/>
+      <c r="L131" s="9" t="n"/>
+    </row>
+    <row r="132" ht="30" customHeight="1">
+      <c r="A132" s="11" t="n">
+        <v>110</v>
+      </c>
+      <c r="B132" s="12" t="inlineStr">
+        <is>
+          <t>ООО «ИРИБ»</t>
+        </is>
+      </c>
+      <c r="C132" s="12" t="inlineStr">
+        <is>
+          <t>Ириб</t>
+        </is>
+      </c>
+      <c r="D132" s="12" t="inlineStr">
+        <is>
+          <t>Нектар</t>
+        </is>
+      </c>
+      <c r="E132" s="12" t="inlineStr">
+        <is>
+          <t>Нектар Ириб Абрикосовый, 3 л, ПЭТ</t>
+        </is>
+      </c>
+      <c r="F132" s="12" t="inlineStr">
+        <is>
+          <t>Абрикосовый</t>
+        </is>
+      </c>
+      <c r="G132" s="11" t="inlineStr">
+        <is>
+          <t>3 л</t>
+        </is>
+      </c>
+      <c r="H132" s="11" t="inlineStr">
+        <is>
+          <t>ПЭТ</t>
+        </is>
+      </c>
+      <c r="I132" s="12" t="inlineStr">
+        <is>
+          <t>IRIB-NEKTAR-ABRIKOSOVYY-3000-PET</t>
+        </is>
+      </c>
+      <c r="J132" s="12" t="inlineStr">
+        <is>
+          <t>Ириб Абрикосовый — фруктовый нектар в ПЭТ-бутылке.</t>
+        </is>
+      </c>
+      <c r="K132" s="13" t="n"/>
+      <c r="L132" s="12" t="n"/>
+    </row>
+    <row r="133" ht="30" customHeight="1">
+      <c r="A133" s="8" t="n">
+        <v>111</v>
+      </c>
+      <c r="B133" s="9" t="inlineStr">
+        <is>
+          <t>ООО «ИРИБ»</t>
+        </is>
+      </c>
+      <c r="C133" s="9" t="inlineStr">
+        <is>
+          <t>Ириб</t>
+        </is>
+      </c>
+      <c r="D133" s="9" t="inlineStr">
+        <is>
+          <t>Нектар</t>
+        </is>
+      </c>
+      <c r="E133" s="9" t="inlineStr">
+        <is>
+          <t>Нектар Ириб Вишневый, 500 мл, стекло</t>
+        </is>
+      </c>
+      <c r="F133" s="9" t="inlineStr">
+        <is>
+          <t>Вишневый</t>
+        </is>
+      </c>
+      <c r="G133" s="8" t="inlineStr">
+        <is>
+          <t>500 мл</t>
+        </is>
+      </c>
+      <c r="H133" s="8" t="inlineStr">
+        <is>
+          <t>стекло</t>
+        </is>
+      </c>
+      <c r="I133" s="9" t="inlineStr">
+        <is>
+          <t>IRIB-NEKTAR-VISHNEVYY-500-GLASS</t>
+        </is>
+      </c>
+      <c r="J133" s="9" t="inlineStr">
+        <is>
+          <t>Ириб Вишневый — фруктовый нектар в стеклянной бутылке.</t>
+        </is>
+      </c>
+      <c r="K133" s="10" t="n"/>
+      <c r="L133" s="9" t="n"/>
+    </row>
+    <row r="134" ht="30" customHeight="1">
+      <c r="A134" s="11" t="n">
+        <v>112</v>
+      </c>
+      <c r="B134" s="12" t="inlineStr">
+        <is>
+          <t>ООО «ИРИБ»</t>
+        </is>
+      </c>
+      <c r="C134" s="12" t="inlineStr">
+        <is>
+          <t>Ириб</t>
+        </is>
+      </c>
+      <c r="D134" s="12" t="inlineStr">
+        <is>
+          <t>Нектар</t>
+        </is>
+      </c>
+      <c r="E134" s="12" t="inlineStr">
+        <is>
+          <t>Нектар Ириб Манговый, 500 мл, стекло</t>
+        </is>
+      </c>
+      <c r="F134" s="12" t="inlineStr">
+        <is>
+          <t>Манговый</t>
+        </is>
+      </c>
+      <c r="G134" s="11" t="inlineStr">
+        <is>
+          <t>500 мл</t>
+        </is>
+      </c>
+      <c r="H134" s="11" t="inlineStr">
+        <is>
+          <t>стекло</t>
+        </is>
+      </c>
+      <c r="I134" s="12" t="inlineStr">
+        <is>
+          <t>IRIB-NEKTAR-MANGOVYY-500-GLASS</t>
+        </is>
+      </c>
+      <c r="J134" s="12" t="inlineStr">
+        <is>
+          <t>Ириб Манговый — фруктовый нектар в стеклянной бутылке.</t>
+        </is>
+      </c>
+      <c r="K134" s="13" t="n"/>
+      <c r="L134" s="12" t="n"/>
+    </row>
+    <row r="135" ht="30" customHeight="1">
+      <c r="A135" s="8" t="n">
+        <v>113</v>
+      </c>
+      <c r="B135" s="9" t="inlineStr">
+        <is>
+          <t>ООО «ИРИБ»</t>
+        </is>
+      </c>
+      <c r="C135" s="9" t="inlineStr">
+        <is>
+          <t>Ириб</t>
+        </is>
+      </c>
+      <c r="D135" s="9" t="inlineStr">
+        <is>
+          <t>Нектар</t>
+        </is>
+      </c>
+      <c r="E135" s="9" t="inlineStr">
+        <is>
+          <t>Нектар Ириб Персиковый, 500 мл, стекло</t>
+        </is>
+      </c>
+      <c r="F135" s="9" t="inlineStr">
+        <is>
+          <t>Персиковый</t>
+        </is>
+      </c>
+      <c r="G135" s="8" t="inlineStr">
+        <is>
+          <t>500 мл</t>
+        </is>
+      </c>
+      <c r="H135" s="8" t="inlineStr">
+        <is>
+          <t>стекло</t>
+        </is>
+      </c>
+      <c r="I135" s="9" t="inlineStr">
+        <is>
+          <t>IRIB-NEKTAR-PERSIKOVYY-500-GLASS</t>
+        </is>
+      </c>
+      <c r="J135" s="9" t="inlineStr">
+        <is>
+          <t>Ириб Персиковый — фруктовый нектар в стеклянной бутылке.</t>
+        </is>
+      </c>
+      <c r="K135" s="10" t="n"/>
+      <c r="L135" s="9" t="n"/>
+    </row>
+    <row r="136" ht="30" customHeight="1">
+      <c r="A136" s="11" t="n">
+        <v>114</v>
+      </c>
+      <c r="B136" s="12" t="inlineStr">
+        <is>
+          <t>ООО «ИРИБ»</t>
+        </is>
+      </c>
+      <c r="C136" s="12" t="inlineStr">
+        <is>
+          <t>Ириб</t>
+        </is>
+      </c>
+      <c r="D136" s="12" t="inlineStr">
+        <is>
+          <t>Нектар</t>
+        </is>
+      </c>
+      <c r="E136" s="12" t="inlineStr">
+        <is>
+          <t>Нектар Ириб Яблочно-абрикосовый, 500 мл, стекло</t>
+        </is>
+      </c>
+      <c r="F136" s="12" t="inlineStr">
+        <is>
+          <t>Яблочно-абрикосовый</t>
+        </is>
+      </c>
+      <c r="G136" s="11" t="inlineStr">
+        <is>
+          <t>500 мл</t>
+        </is>
+      </c>
+      <c r="H136" s="11" t="inlineStr">
+        <is>
+          <t>стекло</t>
+        </is>
+      </c>
+      <c r="I136" s="12" t="inlineStr">
+        <is>
+          <t>IRIB-NEKTAR-YABLOCHNO-ABRIKOSOVYY-500-GLASS</t>
+        </is>
+      </c>
+      <c r="J136" s="12" t="inlineStr">
+        <is>
+          <t>Ириб Яблочно-абрикосовый — фруктовый нектар в стеклянной бутылке.</t>
+        </is>
+      </c>
+      <c r="K136" s="13" t="n"/>
+      <c r="L136" s="12" t="n"/>
+    </row>
+    <row r="137" ht="30" customHeight="1">
+      <c r="A137" s="8" t="n">
+        <v>115</v>
+      </c>
+      <c r="B137" s="9" t="inlineStr">
+        <is>
+          <t>ООО «ИРИБ»</t>
+        </is>
+      </c>
+      <c r="C137" s="9" t="inlineStr">
+        <is>
+          <t>Ириб</t>
+        </is>
+      </c>
+      <c r="D137" s="9" t="inlineStr">
+        <is>
+          <t>Нектар</t>
+        </is>
+      </c>
+      <c r="E137" s="9" t="inlineStr">
+        <is>
+          <t>Нектар Ириб Яблочно-абрикосовый, 3 л, ПЭТ</t>
+        </is>
+      </c>
+      <c r="F137" s="9" t="inlineStr">
+        <is>
+          <t>Яблочно-абрикосовый</t>
+        </is>
+      </c>
+      <c r="G137" s="8" t="inlineStr">
+        <is>
+          <t>3 л</t>
+        </is>
+      </c>
+      <c r="H137" s="8" t="inlineStr">
+        <is>
+          <t>ПЭТ</t>
+        </is>
+      </c>
+      <c r="I137" s="9" t="inlineStr">
+        <is>
+          <t>IRIB-NEKTAR-YABLOCHNO-ABRIKOSOVYY-3000-PET</t>
+        </is>
+      </c>
+      <c r="J137" s="9" t="inlineStr">
+        <is>
+          <t>Ириб Яблочно-абрикосовый — фруктовый нектар в ПЭТ-бутылке.</t>
+        </is>
+      </c>
+      <c r="K137" s="10" t="n"/>
+      <c r="L137" s="9" t="n"/>
+    </row>
+    <row r="138" ht="30" customHeight="1">
+      <c r="A138" s="11" t="n">
+        <v>116</v>
+      </c>
+      <c r="B138" s="12" t="inlineStr">
+        <is>
+          <t>ООО «ИРИБ»</t>
+        </is>
+      </c>
+      <c r="C138" s="12" t="inlineStr">
+        <is>
+          <t>Ириб</t>
+        </is>
+      </c>
+      <c r="D138" s="12" t="inlineStr">
+        <is>
+          <t>Нектар</t>
+        </is>
+      </c>
+      <c r="E138" s="12" t="inlineStr">
+        <is>
+          <t>Нектар Ириб Яблочный, 500 мл, стекло</t>
+        </is>
+      </c>
+      <c r="F138" s="12" t="inlineStr">
+        <is>
+          <t>Яблочный</t>
+        </is>
+      </c>
+      <c r="G138" s="11" t="inlineStr">
+        <is>
+          <t>500 мл</t>
+        </is>
+      </c>
+      <c r="H138" s="11" t="inlineStr">
+        <is>
+          <t>стекло</t>
+        </is>
+      </c>
+      <c r="I138" s="12" t="inlineStr">
+        <is>
+          <t>IRIB-NEKTAR-YABLOCHNYY-500-GLASS</t>
+        </is>
+      </c>
+      <c r="J138" s="12" t="inlineStr">
+        <is>
+          <t>Ириб Яблочный — фруктовый нектар в стеклянной бутылке.</t>
+        </is>
+      </c>
+      <c r="K138" s="13" t="n"/>
+      <c r="L138" s="12" t="n"/>
+    </row>
+    <row r="139" ht="30" customHeight="1">
+      <c r="A139" s="8" t="n">
+        <v>117</v>
+      </c>
+      <c r="B139" s="9" t="inlineStr">
+        <is>
+          <t>ООО «ИРИБ»</t>
+        </is>
+      </c>
+      <c r="C139" s="9" t="inlineStr">
+        <is>
+          <t>Ириб</t>
+        </is>
+      </c>
+      <c r="D139" s="9" t="inlineStr">
+        <is>
+          <t>Нектар</t>
+        </is>
+      </c>
+      <c r="E139" s="9" t="inlineStr">
+        <is>
+          <t>Нектар Ириб Яблочный, 750 мл, стекло</t>
+        </is>
+      </c>
+      <c r="F139" s="9" t="inlineStr">
+        <is>
+          <t>Яблочный</t>
+        </is>
+      </c>
+      <c r="G139" s="8" t="inlineStr">
+        <is>
+          <t>750 мл</t>
+        </is>
+      </c>
+      <c r="H139" s="8" t="inlineStr">
+        <is>
+          <t>стекло</t>
+        </is>
+      </c>
+      <c r="I139" s="9" t="inlineStr">
+        <is>
+          <t>IRIB-NEKTAR-YABLOCHNYY-750-GLASS</t>
+        </is>
+      </c>
+      <c r="J139" s="9" t="inlineStr">
+        <is>
+          <t>Ириб Яблочный — фруктовый нектар в стеклянной бутылке.</t>
+        </is>
+      </c>
+      <c r="K139" s="10" t="n"/>
+      <c r="L139" s="9" t="n"/>
+    </row>
+    <row r="140" ht="30" customHeight="1">
+      <c r="A140" s="11" t="n">
+        <v>118</v>
+      </c>
+      <c r="B140" s="12" t="inlineStr">
+        <is>
+          <t>ООО «ИРИБ»</t>
+        </is>
+      </c>
+      <c r="C140" s="12" t="inlineStr">
+        <is>
+          <t>Ириб</t>
+        </is>
+      </c>
+      <c r="D140" s="12" t="inlineStr">
+        <is>
+          <t>Нектар</t>
+        </is>
+      </c>
+      <c r="E140" s="12" t="inlineStr">
+        <is>
+          <t>Нектар Ириб Яблочный, 3 л, ПЭТ</t>
+        </is>
+      </c>
+      <c r="F140" s="12" t="inlineStr">
+        <is>
+          <t>Яблочный</t>
+        </is>
+      </c>
+      <c r="G140" s="11" t="inlineStr">
+        <is>
+          <t>3 л</t>
+        </is>
+      </c>
+      <c r="H140" s="11" t="inlineStr">
+        <is>
+          <t>ПЭТ</t>
+        </is>
+      </c>
+      <c r="I140" s="12" t="inlineStr">
+        <is>
+          <t>IRIB-NEKTAR-YABLOCHNYY-3000-PET</t>
+        </is>
+      </c>
+      <c r="J140" s="12" t="inlineStr">
+        <is>
+          <t>Ириб Яблочный — фруктовый нектар в ПЭТ-бутылке.</t>
+        </is>
+      </c>
+      <c r="K140" s="13" t="n"/>
+      <c r="L140" s="12" t="n"/>
+    </row>
+    <row r="141" ht="30" customHeight="1">
+      <c r="A141" s="8" t="n">
+        <v>119</v>
+      </c>
+      <c r="B141" s="9" t="inlineStr"/>
+      <c r="C141" s="9" t="inlineStr">
+        <is>
+          <t>Ириб</t>
+        </is>
+      </c>
+      <c r="D141" s="9" t="inlineStr">
+        <is>
+          <t>Нектар</t>
+        </is>
+      </c>
+      <c r="E141" s="9" t="inlineStr">
+        <is>
+          <t>Нектар Ириб ст/б 0,75л Абрикосовый</t>
+        </is>
+      </c>
+      <c r="F141" s="9" t="inlineStr">
+        <is>
+          <t>Абрикосовый</t>
+        </is>
+      </c>
+      <c r="G141" s="8" t="inlineStr">
+        <is>
+          <t>750 мл</t>
+        </is>
+      </c>
+      <c r="H141" s="8" t="inlineStr">
+        <is>
+          <t>стекло</t>
+        </is>
+      </c>
+      <c r="I141" s="9" t="inlineStr">
+        <is>
+          <t>ZY-IRIB-750-GLASS-002</t>
+        </is>
+      </c>
+      <c r="J141" s="9" t="inlineStr">
+        <is>
+          <t>Ириб Абрикосовый — фруктовый нектар в стеклянной бутылке.</t>
+        </is>
+      </c>
+      <c r="K141" s="10" t="n"/>
+      <c r="L141" s="9" t="n"/>
+    </row>
+    <row r="142" ht="30" customHeight="1">
+      <c r="A142" s="11" t="n">
+        <v>120</v>
+      </c>
+      <c r="B142" s="12" t="inlineStr"/>
+      <c r="C142" s="12" t="inlineStr">
+        <is>
+          <t>Ириб</t>
+        </is>
+      </c>
+      <c r="D142" s="12" t="inlineStr">
+        <is>
+          <t>Нектар</t>
+        </is>
+      </c>
+      <c r="E142" s="12" t="inlineStr">
+        <is>
+          <t>Нектар Ириб ст/б 0,75л Вишневый 50%</t>
+        </is>
+      </c>
+      <c r="F142" s="12" t="inlineStr">
+        <is>
+          <t>Вишневый</t>
+        </is>
+      </c>
+      <c r="G142" s="11" t="inlineStr">
+        <is>
+          <t>750 мл</t>
+        </is>
+      </c>
+      <c r="H142" s="11" t="inlineStr">
+        <is>
+          <t>стекло</t>
+        </is>
+      </c>
+      <c r="I142" s="12" t="inlineStr">
+        <is>
+          <t>ZY-IRIB-750-GLASS-004</t>
+        </is>
+      </c>
+      <c r="J142" s="12" t="inlineStr">
+        <is>
+          <t>Ириб Вишневый — фруктовый нектар в стеклянной бутылке.</t>
+        </is>
+      </c>
+      <c r="K142" s="13" t="n"/>
+      <c r="L142" s="12" t="n"/>
+    </row>
+    <row r="143" ht="30" customHeight="1">
+      <c r="A143" s="8" t="n">
+        <v>121</v>
+      </c>
+      <c r="B143" s="9" t="inlineStr"/>
+      <c r="C143" s="9" t="inlineStr">
+        <is>
+          <t>Ириб</t>
+        </is>
+      </c>
+      <c r="D143" s="9" t="inlineStr">
+        <is>
+          <t>Нектар</t>
+        </is>
+      </c>
+      <c r="E143" s="9" t="inlineStr">
+        <is>
+          <t>Нектар Ириб ст/б 0,75л Персиковый 50%</t>
+        </is>
+      </c>
+      <c r="F143" s="9" t="inlineStr">
+        <is>
+          <t>Персиковый</t>
+        </is>
+      </c>
+      <c r="G143" s="8" t="inlineStr">
+        <is>
+          <t>750 мл</t>
+        </is>
+      </c>
+      <c r="H143" s="8" t="inlineStr">
+        <is>
+          <t>стекло</t>
+        </is>
+      </c>
+      <c r="I143" s="9" t="inlineStr">
+        <is>
+          <t>ZY-IRIB-750-GLASS-006</t>
+        </is>
+      </c>
+      <c r="J143" s="9" t="inlineStr">
+        <is>
+          <t>Ириб Персиковый — фруктовый нектар в стеклянной бутылке.</t>
+        </is>
+      </c>
+      <c r="K143" s="10" t="n"/>
+      <c r="L143" s="9" t="n"/>
+    </row>
+    <row r="144" ht="30" customHeight="1">
+      <c r="A144" s="11" t="n">
+        <v>122</v>
+      </c>
+      <c r="B144" s="12" t="inlineStr">
+        <is>
+          <t>ООО «ИРИБ»</t>
+        </is>
+      </c>
+      <c r="C144" s="12" t="inlineStr">
+        <is>
+          <t>Родничок</t>
+        </is>
+      </c>
+      <c r="D144" s="12" t="inlineStr">
+        <is>
+          <t>Питьевая вода</t>
+        </is>
+      </c>
+      <c r="E144" s="12" t="inlineStr">
+        <is>
+          <t>Родничок Негазированная, 330 мл, ПЭТ</t>
+        </is>
+      </c>
+      <c r="F144" s="12" t="inlineStr">
+        <is>
+          <t>Не</t>
+        </is>
+      </c>
+      <c r="G144" s="11" t="inlineStr">
+        <is>
+          <t>330 мл</t>
+        </is>
+      </c>
+      <c r="H144" s="11" t="inlineStr">
+        <is>
+          <t>ПЭТ</t>
+        </is>
+      </c>
+      <c r="I144" s="12" t="inlineStr">
+        <is>
+          <t>IRIB-RODNICHOK-NEGAZIROVANNAYA-330-PET</t>
+        </is>
+      </c>
+      <c r="J144" s="12" t="inlineStr">
+        <is>
+          <t>Негазированная питьевая вода Родничок в ПЭТ-бутылке.</t>
+        </is>
+      </c>
+      <c r="K144" s="13" t="n"/>
+      <c r="L144" s="12" t="n"/>
+    </row>
+    <row r="145" ht="30" customHeight="1">
+      <c r="A145" s="8" t="n">
+        <v>123</v>
+      </c>
+      <c r="B145" s="9" t="inlineStr">
+        <is>
+          <t>ООО «ИРИБ»</t>
+        </is>
+      </c>
+      <c r="C145" s="9" t="inlineStr">
+        <is>
+          <t>Чегери</t>
+        </is>
+      </c>
+      <c r="D145" s="9" t="inlineStr">
+        <is>
+          <t>Питьевая вода</t>
+        </is>
+      </c>
+      <c r="E145" s="9" t="inlineStr">
+        <is>
+          <t>Чегери Негазированная, 500 мл, ПЭТ</t>
+        </is>
+      </c>
+      <c r="F145" s="9" t="inlineStr">
+        <is>
+          <t>Не</t>
+        </is>
+      </c>
+      <c r="G145" s="8" t="inlineStr">
+        <is>
+          <t>500 мл</t>
+        </is>
+      </c>
+      <c r="H145" s="8" t="inlineStr">
+        <is>
+          <t>ПЭТ</t>
+        </is>
+      </c>
+      <c r="I145" s="9" t="inlineStr">
+        <is>
+          <t>IRIB-CHEGERI-NEGAZIROVANNAYA-500-PET</t>
+        </is>
+      </c>
+      <c r="J145" s="9" t="inlineStr">
+        <is>
+          <t>Негазированная питьевая вода Чегери в ПЭТ-бутылке.</t>
+        </is>
+      </c>
+      <c r="K145" s="10" t="n"/>
+      <c r="L145" s="9" t="n"/>
+    </row>
+    <row r="146" ht="30" customHeight="1">
+      <c r="A146" s="11" t="n">
+        <v>124</v>
+      </c>
+      <c r="B146" s="12" t="inlineStr">
+        <is>
+          <t>ООО «ИРИБ»</t>
+        </is>
+      </c>
+      <c r="C146" s="12" t="inlineStr">
+        <is>
+          <t>Родниковая свежесть</t>
+        </is>
+      </c>
+      <c r="D146" s="12" t="inlineStr">
+        <is>
+          <t>Минеральная вода</t>
+        </is>
+      </c>
+      <c r="E146" s="12" t="inlineStr">
+        <is>
+          <t>Родниковая свежесть Негазированная, 19 л, ПЭТ</t>
+        </is>
+      </c>
+      <c r="F146" s="12" t="inlineStr">
+        <is>
+          <t>Не</t>
+        </is>
+      </c>
+      <c r="G146" s="11" t="inlineStr">
+        <is>
+          <t>19 л</t>
+        </is>
+      </c>
+      <c r="H146" s="11" t="inlineStr">
+        <is>
+          <t>ПЭТ</t>
+        </is>
+      </c>
+      <c r="I146" s="12" t="inlineStr">
+        <is>
+          <t>IRIB-RODNIKOVAYA-SVEZHEST-NEGAZIROVANNAYA-19000-PET</t>
+        </is>
+      </c>
+      <c r="J146" s="12" t="inlineStr">
+        <is>
+          <t>Минеральная вода Родниковая свежесть в ПЭТ-бутылке.</t>
+        </is>
+      </c>
+      <c r="K146" s="13" t="n"/>
+      <c r="L146" s="12" t="n"/>
+    </row>
+    <row r="147" ht="30" customHeight="1">
+      <c r="A147" s="8" t="n">
+        <v>125</v>
+      </c>
+      <c r="B147" s="9" t="inlineStr">
+        <is>
+          <t>ООО «ИРИБ»</t>
+        </is>
+      </c>
+      <c r="C147" s="9" t="inlineStr">
+        <is>
+          <t>Талих</t>
+        </is>
+      </c>
+      <c r="D147" s="9" t="inlineStr">
+        <is>
+          <t>Негазированная вода</t>
+        </is>
+      </c>
+      <c r="E147" s="9" t="inlineStr">
+        <is>
+          <t>Вода Талих, 600 мл, ПЭТ</t>
+        </is>
+      </c>
+      <c r="F147" s="9" t="inlineStr">
+        <is>
+          <t>Вода Талих</t>
+        </is>
+      </c>
+      <c r="G147" s="8" t="inlineStr">
+        <is>
+          <t>600 мл</t>
+        </is>
+      </c>
+      <c r="H147" s="8" t="inlineStr">
+        <is>
+          <t>ПЭТ</t>
+        </is>
+      </c>
+      <c r="I147" s="9" t="inlineStr">
+        <is>
+          <t>IRIB-TALIH-NEGAZIROVANNAYA-600-PET</t>
+        </is>
+      </c>
+      <c r="J147" s="9" t="inlineStr">
+        <is>
+          <t>Питьевая вода Талих в ПЭТ-бутылке.</t>
+        </is>
+      </c>
+      <c r="K147" s="10" t="n"/>
+      <c r="L147" s="9" t="n"/>
+    </row>
+    <row r="148" ht="30" customHeight="1">
+      <c r="A148" s="11" t="n">
+        <v>126</v>
+      </c>
+      <c r="B148" s="12" t="inlineStr">
+        <is>
+          <t>ООО «ИРИБ»</t>
+        </is>
+      </c>
+      <c r="C148" s="12" t="inlineStr">
+        <is>
+          <t>Талих</t>
+        </is>
+      </c>
+      <c r="D148" s="12" t="inlineStr">
+        <is>
+          <t>Негазированная вода</t>
+        </is>
+      </c>
+      <c r="E148" s="12" t="inlineStr">
+        <is>
+          <t>Вода Талих, 1,5 л, ПЭТ</t>
+        </is>
+      </c>
+      <c r="F148" s="12" t="inlineStr">
+        <is>
+          <t>Вода Талих</t>
+        </is>
+      </c>
+      <c r="G148" s="11" t="inlineStr">
+        <is>
+          <t>1,5 л</t>
+        </is>
+      </c>
+      <c r="H148" s="11" t="inlineStr">
+        <is>
+          <t>ПЭТ</t>
+        </is>
+      </c>
+      <c r="I148" s="12" t="inlineStr">
+        <is>
+          <t>IRIB-TALIH-NEGAZIROVANNAYA-1500-PET</t>
+        </is>
+      </c>
+      <c r="J148" s="12" t="inlineStr">
+        <is>
+          <t>Питьевая вода Талих в ПЭТ-бутылке.</t>
+        </is>
+      </c>
+      <c r="K148" s="13" t="n"/>
+      <c r="L148" s="12" t="n"/>
+    </row>
+    <row r="149" ht="30" customHeight="1">
+      <c r="A149" s="8" t="n">
+        <v>127</v>
+      </c>
+      <c r="B149" s="9" t="inlineStr">
+        <is>
+          <t>ООО «ИРИБ»</t>
+        </is>
+      </c>
+      <c r="C149" s="9" t="inlineStr">
+        <is>
+          <t>Талих</t>
+        </is>
+      </c>
+      <c r="D149" s="9" t="inlineStr">
+        <is>
+          <t>Негазированная вода</t>
+        </is>
+      </c>
+      <c r="E149" s="9" t="inlineStr">
+        <is>
+          <t>Вода Талих, 5 л, ПЭТ</t>
+        </is>
+      </c>
+      <c r="F149" s="9" t="inlineStr">
+        <is>
+          <t>Вода Талих</t>
+        </is>
+      </c>
+      <c r="G149" s="8" t="inlineStr">
+        <is>
+          <t>5 л</t>
+        </is>
+      </c>
+      <c r="H149" s="8" t="inlineStr">
+        <is>
+          <t>ПЭТ</t>
+        </is>
+      </c>
+      <c r="I149" s="9" t="inlineStr">
+        <is>
+          <t>IRIB-TALIH-NEGAZIROVANNAYA-5000-PET</t>
+        </is>
+      </c>
+      <c r="J149" s="9" t="inlineStr">
+        <is>
+          <t>Питьевая вода Талих в ПЭТ-бутылке.</t>
+        </is>
+      </c>
+      <c r="K149" s="10" t="n"/>
+      <c r="L149" s="9" t="n"/>
+    </row>
+    <row r="150" ht="30" customHeight="1">
+      <c r="A150" s="11" t="n">
+        <v>128</v>
+      </c>
+      <c r="B150" s="12" t="inlineStr"/>
+      <c r="C150" s="12" t="inlineStr">
+        <is>
+          <t>Ириб</t>
+        </is>
+      </c>
+      <c r="D150" s="12" t="inlineStr">
+        <is>
+          <t>Газированная вода</t>
+        </is>
+      </c>
+      <c r="E150" s="12" t="inlineStr">
+        <is>
+          <t>Вода Ириб минер Тарки Тау ст/б 0,5л</t>
+        </is>
+      </c>
+      <c r="F150" s="12" t="inlineStr">
+        <is>
+          <t>Вода Ириб минер Тарки Тау 0</t>
+        </is>
+      </c>
+      <c r="G150" s="11" t="inlineStr">
+        <is>
+          <t>500 мл</t>
+        </is>
+      </c>
+      <c r="H150" s="11" t="inlineStr">
+        <is>
+          <t>стекло</t>
+        </is>
+      </c>
+      <c r="I150" s="12" t="inlineStr">
+        <is>
+          <t>ZY-IRIB-500-GLASS-001</t>
+        </is>
+      </c>
+      <c r="J150" s="12" t="inlineStr">
+        <is>
+          <t>Минеральная вода Ириб в стеклянной бутылке.</t>
+        </is>
+      </c>
+      <c r="K150" s="13" t="n"/>
+      <c r="L150" s="12" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A11:L100"/>
-  <mergeCells count="12">
+  <autoFilter ref="A11:L150"/>
+  <mergeCells count="13">
     <mergeCell ref="A26:L26"/>
     <mergeCell ref="A24:L24"/>
+    <mergeCell ref="A101:L101"/>
     <mergeCell ref="A60:L60"/>
     <mergeCell ref="B2:F2"/>
     <mergeCell ref="A33:L33"/>

</xml_diff>